<commit_message>
Restore 5-column local Excel format and refresh all output data
Match the user's fund-filing-scraper template: single Sheet1 with
产品名称/托管行/产品类型/报会日期/是否已发行 only. Re-collect data with
fixed report dates and custodian/issued logic.

Co-authored-by: linzhuoran79 <linzhuoran79@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/易方达_广发_验证渠道_2025-2026Q1.xlsx
+++ b/output/易方达_广发_验证渠道_2025-2026Q1.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="验证渠道" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="数据质量检查" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -611,7 +610,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>广发中证800指数增强型证券投资基金 | 报会日期 2025-01-08</t>
+          <t>广发中证智选高股息策略交易型开放式指数证券投资基金 | 报会日期 2025-01-07</t>
         </is>
       </c>
     </row>
@@ -633,7 +632,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>广发中证智选高股息策略交易型开放式指数证券投资基金 | 报会日期 2025-01-07</t>
+          <t>广发中证800指数增强型证券投资基金 | 报会日期 2025-01-08</t>
         </is>
       </c>
     </row>
@@ -766,372 +765,6 @@
       <c r="D16" t="inlineStr">
         <is>
           <t>广发科技智选股票型发起式证券投资基金 | 首发区间 2025-04-01 至 2025-04-15</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>问题类型</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>产品名称</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>当前值</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>广发中证A500指数增强型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2025-01-02 至 2025-01-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>广发产业甄选混合型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2025-01-02 至 2025-01-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>广发同远回报混合型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2025-03-03 至 2025-03-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>广发上证科创板100交易型开放式指数证券投资基金</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2025-04-30 至 2025-06-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>广发悦康三个月持有期混合型基金中基金（FOF）</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2025-09-26 至 2025-12-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>广发集辉债券型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2025-11-24 至 2025-12-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>广发添益120天滚动持有债券型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-02-02 至 2026-02-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>易方达上证基准做市公司债交易型开放式指数证券投资基金</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2025-01-07 至 2025-01-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>易方达上证180交易型开放式指数证券投资基金联接基金</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2025-01-13 至 2025-01-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>易方达稳裕120天滚动持有债券型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2025-02-17 至 2025-02-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>易方达安旭90天持有期债券型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2025-04-21 至 2025-04-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>易方达高股息量化选股股票型发起式证券投资基金</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2025-04-21 至 2025-04-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>易方达养老目标日期2060五年持有期混合型发起式基金中基金（FOF）</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2025-06-09 至 2025-09-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>易方达中证A50增强策略交易型开放式指数证券投资基金</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2025-06-16 至 2025-09-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>首发无对应报会记录</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>易方达安如30天持有期债券型证券投资基金</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>可能是变更注册、跨期报会或名称匹配未命中。</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2025-07-14 至 2025-07-25</t>
         </is>
       </c>
     </row>

</xml_diff>